<commit_message>
att dia 08 e 09
</commit_message>
<xml_diff>
--- a/primeirasemanasetembro.xlsx
+++ b/primeirasemanasetembro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivina\Desktop\jogodobicho\jogodobicho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5910E270-C306-413C-941C-CAB0BDAEB35F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C8F5002-55DF-4743-8D4D-92C19096E0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{500AFD6E-13E7-4543-8FDB-D63E104D29D0}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185FBA4-3391-45B3-811A-4861B6CE3709}">
-  <dimension ref="A1:T2181"/>
+  <dimension ref="A1:T2211"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.44140625" customWidth="1"/>
@@ -38418,6 +38418,486 @@
         <v>8</v>
       </c>
     </row>
+    <row r="2182" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2182">
+        <v>110</v>
+      </c>
+      <c r="B2182" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2182">
+        <v>0</v>
+      </c>
+      <c r="D2182">
+        <v>5714</v>
+      </c>
+      <c r="E2182">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2183" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2183">
+        <v>110</v>
+      </c>
+      <c r="B2183" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2183">
+        <v>0</v>
+      </c>
+      <c r="D2183">
+        <v>5336</v>
+      </c>
+      <c r="E2183">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2184" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2184">
+        <v>110</v>
+      </c>
+      <c r="B2184" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2184">
+        <v>0</v>
+      </c>
+      <c r="D2184">
+        <v>8238</v>
+      </c>
+      <c r="E2184">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2185" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2185">
+        <v>110</v>
+      </c>
+      <c r="B2185" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2185">
+        <v>0</v>
+      </c>
+      <c r="D2185">
+        <v>9191</v>
+      </c>
+      <c r="E2185">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2186" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2186">
+        <v>110</v>
+      </c>
+      <c r="B2186" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2186">
+        <v>0</v>
+      </c>
+      <c r="D2186">
+        <v>4249</v>
+      </c>
+      <c r="E2186">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2187" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2187">
+        <v>110</v>
+      </c>
+      <c r="B2187" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2187">
+        <v>0</v>
+      </c>
+      <c r="D2187">
+        <v>9761</v>
+      </c>
+      <c r="E2187">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2188" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2188">
+        <v>110</v>
+      </c>
+      <c r="B2188" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2188">
+        <v>0</v>
+      </c>
+      <c r="D2188">
+        <v>3937</v>
+      </c>
+      <c r="E2188">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2189" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2189">
+        <v>110</v>
+      </c>
+      <c r="B2189" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2189">
+        <v>0</v>
+      </c>
+      <c r="D2189">
+        <v>5711</v>
+      </c>
+      <c r="E2189">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2190" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2190">
+        <v>110</v>
+      </c>
+      <c r="B2190" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2190">
+        <v>0</v>
+      </c>
+      <c r="D2190">
+        <v>9283</v>
+      </c>
+      <c r="E2190">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2191" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2191">
+        <v>110</v>
+      </c>
+      <c r="B2191" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2191">
+        <v>0</v>
+      </c>
+      <c r="D2191">
+        <v>8792</v>
+      </c>
+      <c r="E2191">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2192" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2192">
+        <v>110</v>
+      </c>
+      <c r="B2192" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2192">
+        <v>1</v>
+      </c>
+      <c r="D2192">
+        <v>2558</v>
+      </c>
+      <c r="E2192">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2193">
+        <v>110</v>
+      </c>
+      <c r="B2193" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2193">
+        <v>1</v>
+      </c>
+      <c r="D2193">
+        <v>6989</v>
+      </c>
+      <c r="E2193">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2194" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2194">
+        <v>110</v>
+      </c>
+      <c r="B2194" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2194">
+        <v>1</v>
+      </c>
+      <c r="D2194">
+        <v>5078</v>
+      </c>
+      <c r="E2194">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2195">
+        <v>110</v>
+      </c>
+      <c r="B2195" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2195">
+        <v>1</v>
+      </c>
+      <c r="D2195">
+        <v>3184</v>
+      </c>
+      <c r="E2195">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2196">
+        <v>110</v>
+      </c>
+      <c r="B2196" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2196">
+        <v>1</v>
+      </c>
+      <c r="D2196">
+        <v>3454</v>
+      </c>
+      <c r="E2196">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2197">
+        <v>110</v>
+      </c>
+      <c r="B2197" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2197">
+        <v>1</v>
+      </c>
+      <c r="D2197">
+        <v>1188</v>
+      </c>
+      <c r="E2197">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2198">
+        <v>110</v>
+      </c>
+      <c r="B2198" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2198">
+        <v>1</v>
+      </c>
+      <c r="D2198">
+        <v>2243</v>
+      </c>
+      <c r="E2198">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2199">
+        <v>110</v>
+      </c>
+      <c r="B2199" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2199">
+        <v>1</v>
+      </c>
+      <c r="D2199">
+        <v>4365</v>
+      </c>
+      <c r="E2199">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2200">
+        <v>110</v>
+      </c>
+      <c r="B2200" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2200">
+        <v>1</v>
+      </c>
+      <c r="D2200">
+        <v>6547</v>
+      </c>
+      <c r="E2200">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2201">
+        <v>110</v>
+      </c>
+      <c r="B2201" s="10">
+        <v>46030</v>
+      </c>
+      <c r="C2201">
+        <v>1</v>
+      </c>
+      <c r="D2201">
+        <v>6376</v>
+      </c>
+      <c r="E2201">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2202" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2202">
+        <v>0</v>
+      </c>
+      <c r="D2202">
+        <v>2720</v>
+      </c>
+      <c r="E2202">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2203" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2203">
+        <v>0</v>
+      </c>
+      <c r="D2203">
+        <v>6449</v>
+      </c>
+      <c r="E2203">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2204" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2204">
+        <v>0</v>
+      </c>
+      <c r="D2204">
+        <v>4735</v>
+      </c>
+      <c r="E2204">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2205" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2205" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2205">
+        <v>0</v>
+      </c>
+      <c r="D2205">
+        <v>343</v>
+      </c>
+      <c r="E2205">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2206" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2206" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2206">
+        <v>0</v>
+      </c>
+      <c r="D2206">
+        <v>8468</v>
+      </c>
+      <c r="E2206">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2207" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2207" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2207">
+        <v>0</v>
+      </c>
+      <c r="D2207">
+        <v>3501</v>
+      </c>
+      <c r="E2207">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2208" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2208" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2208">
+        <v>0</v>
+      </c>
+      <c r="D2208">
+        <v>48</v>
+      </c>
+      <c r="E2208">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2209" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B2209" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2209">
+        <v>0</v>
+      </c>
+      <c r="D2209">
+        <v>2313</v>
+      </c>
+      <c r="E2209">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2210" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B2210" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2210">
+        <v>0</v>
+      </c>
+      <c r="D2210">
+        <v>62</v>
+      </c>
+      <c r="E2210">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2211" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B2211" s="10">
+        <v>46031</v>
+      </c>
+      <c r="C2211">
+        <v>0</v>
+      </c>
+      <c r="D2211">
+        <v>7512</v>
+      </c>
+      <c r="E2211">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
att dia 10 e pulando a previsao do domingo
</commit_message>
<xml_diff>
--- a/primeirasemanasetembro.xlsx
+++ b/primeirasemanasetembro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivina\Desktop\jogodobicho\jogodobicho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA6F64F-81E5-4FDE-B8C7-8D71396140C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8F07BA-ABB1-40F6-8185-73FC5A78C110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{500AFD6E-13E7-4543-8FDB-D63E104D29D0}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185FBA4-3391-45B3-811A-4861B6CE3709}">
-  <dimension ref="A1:T2231"/>
+  <dimension ref="A1:T2241"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.44140625" customWidth="1"/>
@@ -39268,6 +39268,176 @@
         <v>20</v>
       </c>
     </row>
+    <row r="2232" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2232">
+        <v>112</v>
+      </c>
+      <c r="B2232" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2232">
+        <v>1</v>
+      </c>
+      <c r="D2232">
+        <v>7551</v>
+      </c>
+      <c r="E2232">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2233" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2233">
+        <v>112</v>
+      </c>
+      <c r="B2233" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2233">
+        <v>1</v>
+      </c>
+      <c r="D2233">
+        <v>4285</v>
+      </c>
+      <c r="E2233">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2234" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2234">
+        <v>112</v>
+      </c>
+      <c r="B2234" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2234">
+        <v>1</v>
+      </c>
+      <c r="D2234">
+        <v>2375</v>
+      </c>
+      <c r="E2234">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2235" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2235">
+        <v>112</v>
+      </c>
+      <c r="B2235" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2235">
+        <v>1</v>
+      </c>
+      <c r="D2235">
+        <v>1154</v>
+      </c>
+      <c r="E2235">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2236" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2236">
+        <v>112</v>
+      </c>
+      <c r="B2236" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2236">
+        <v>1</v>
+      </c>
+      <c r="D2236">
+        <v>3701</v>
+      </c>
+      <c r="E2236">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2237" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2237">
+        <v>112</v>
+      </c>
+      <c r="B2237" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2237">
+        <v>1</v>
+      </c>
+      <c r="D2237">
+        <v>5620</v>
+      </c>
+      <c r="E2237">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2238" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2238">
+        <v>112</v>
+      </c>
+      <c r="B2238" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2238">
+        <v>1</v>
+      </c>
+      <c r="D2238">
+        <v>2035</v>
+      </c>
+      <c r="E2238">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2239" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2239">
+        <v>112</v>
+      </c>
+      <c r="B2239" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2239">
+        <v>1</v>
+      </c>
+      <c r="D2239">
+        <v>3947</v>
+      </c>
+      <c r="E2239">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2240" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2240">
+        <v>112</v>
+      </c>
+      <c r="B2240" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2240">
+        <v>1</v>
+      </c>
+      <c r="D2240">
+        <v>5101</v>
+      </c>
+      <c r="E2240">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2241" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2241">
+        <v>112</v>
+      </c>
+      <c r="B2241" s="10">
+        <v>46032</v>
+      </c>
+      <c r="C2241">
+        <v>1</v>
+      </c>
+      <c r="D2241">
+        <v>3236</v>
+      </c>
+      <c r="E2241">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
att dia 12 - 13
</commit_message>
<xml_diff>
--- a/primeirasemanasetembro.xlsx
+++ b/primeirasemanasetembro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivina\Desktop\jogodobicho\jogodobicho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8F07BA-ABB1-40F6-8185-73FC5A78C110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F30D9F-FC81-4BF1-810C-2975851856AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{500AFD6E-13E7-4543-8FDB-D63E104D29D0}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185FBA4-3391-45B3-811A-4861B6CE3709}">
-  <dimension ref="A1:T2241"/>
+  <dimension ref="A1:T2281"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.44140625" customWidth="1"/>
@@ -39438,6 +39438,686 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2242" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2242">
+        <v>113</v>
+      </c>
+      <c r="B2242" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2242">
+        <v>0</v>
+      </c>
+      <c r="D2242">
+        <v>4001</v>
+      </c>
+      <c r="E2242">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2243" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2243">
+        <v>113</v>
+      </c>
+      <c r="B2243" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2243">
+        <v>0</v>
+      </c>
+      <c r="D2243">
+        <v>2380</v>
+      </c>
+      <c r="E2243">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2244" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2244">
+        <v>113</v>
+      </c>
+      <c r="B2244" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2244">
+        <v>0</v>
+      </c>
+      <c r="D2244">
+        <v>9206</v>
+      </c>
+      <c r="E2244">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2245" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2245">
+        <v>113</v>
+      </c>
+      <c r="B2245" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2245">
+        <v>0</v>
+      </c>
+      <c r="D2245">
+        <v>452</v>
+      </c>
+      <c r="E2245">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2246" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2246">
+        <v>113</v>
+      </c>
+      <c r="B2246" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2246">
+        <v>0</v>
+      </c>
+      <c r="D2246">
+        <v>2836</v>
+      </c>
+      <c r="E2246">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2247" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2247">
+        <v>113</v>
+      </c>
+      <c r="B2247" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2247">
+        <v>0</v>
+      </c>
+      <c r="D2247">
+        <v>252</v>
+      </c>
+      <c r="E2247">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2248" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2248">
+        <v>113</v>
+      </c>
+      <c r="B2248" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2248">
+        <v>0</v>
+      </c>
+      <c r="D2248">
+        <v>1006</v>
+      </c>
+      <c r="E2248">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2249" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2249">
+        <v>113</v>
+      </c>
+      <c r="B2249" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2249">
+        <v>0</v>
+      </c>
+      <c r="D2249">
+        <v>4915</v>
+      </c>
+      <c r="E2249">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2250" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2250">
+        <v>113</v>
+      </c>
+      <c r="B2250" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2250">
+        <v>0</v>
+      </c>
+      <c r="D2250">
+        <v>5471</v>
+      </c>
+      <c r="E2250">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2251" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2251">
+        <v>113</v>
+      </c>
+      <c r="B2251" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2251">
+        <v>0</v>
+      </c>
+      <c r="D2251">
+        <v>7246</v>
+      </c>
+      <c r="E2251">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2252" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2252">
+        <v>113</v>
+      </c>
+      <c r="B2252" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2252">
+        <v>1</v>
+      </c>
+      <c r="D2252">
+        <v>9385</v>
+      </c>
+      <c r="E2252">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2253" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2253">
+        <v>113</v>
+      </c>
+      <c r="B2253" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2253">
+        <v>1</v>
+      </c>
+      <c r="D2253">
+        <v>5385</v>
+      </c>
+      <c r="E2253">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2254" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2254">
+        <v>113</v>
+      </c>
+      <c r="B2254" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2254">
+        <v>1</v>
+      </c>
+      <c r="D2254">
+        <v>6732</v>
+      </c>
+      <c r="E2254">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2255" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2255">
+        <v>113</v>
+      </c>
+      <c r="B2255" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2255">
+        <v>1</v>
+      </c>
+      <c r="D2255">
+        <v>1909</v>
+      </c>
+      <c r="E2255">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2256" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2256">
+        <v>113</v>
+      </c>
+      <c r="B2256" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2256">
+        <v>1</v>
+      </c>
+      <c r="D2256">
+        <v>696</v>
+      </c>
+      <c r="E2256">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2257" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2257">
+        <v>113</v>
+      </c>
+      <c r="B2257" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2257">
+        <v>1</v>
+      </c>
+      <c r="D2257">
+        <v>9995</v>
+      </c>
+      <c r="E2257">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2258" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2258">
+        <v>113</v>
+      </c>
+      <c r="B2258" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2258">
+        <v>1</v>
+      </c>
+      <c r="D2258">
+        <v>8303</v>
+      </c>
+      <c r="E2258">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2259" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2259">
+        <v>113</v>
+      </c>
+      <c r="B2259" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2259">
+        <v>1</v>
+      </c>
+      <c r="D2259">
+        <v>3991</v>
+      </c>
+      <c r="E2259">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2260" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2260">
+        <v>113</v>
+      </c>
+      <c r="B2260" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2260">
+        <v>1</v>
+      </c>
+      <c r="D2260">
+        <v>7189</v>
+      </c>
+      <c r="E2260">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2261" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2261">
+        <v>113</v>
+      </c>
+      <c r="B2261" s="10">
+        <v>46034</v>
+      </c>
+      <c r="C2261">
+        <v>1</v>
+      </c>
+      <c r="D2261">
+        <v>4090</v>
+      </c>
+      <c r="E2261">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2262" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2262">
+        <v>114</v>
+      </c>
+      <c r="B2262" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2262">
+        <v>0</v>
+      </c>
+      <c r="D2262">
+        <v>3777</v>
+      </c>
+      <c r="E2262">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2263" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2263">
+        <v>114</v>
+      </c>
+      <c r="B2263" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2263">
+        <v>0</v>
+      </c>
+      <c r="D2263">
+        <v>550</v>
+      </c>
+      <c r="E2263">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2264" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2264">
+        <v>114</v>
+      </c>
+      <c r="B2264" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2264">
+        <v>0</v>
+      </c>
+      <c r="D2264">
+        <v>8260</v>
+      </c>
+      <c r="E2264">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2265" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2265">
+        <v>114</v>
+      </c>
+      <c r="B2265" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2265">
+        <v>0</v>
+      </c>
+      <c r="D2265">
+        <v>9425</v>
+      </c>
+      <c r="E2265">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2266" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2266">
+        <v>114</v>
+      </c>
+      <c r="B2266" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2266">
+        <v>0</v>
+      </c>
+      <c r="D2266">
+        <v>7948</v>
+      </c>
+      <c r="E2266">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2267" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2267">
+        <v>114</v>
+      </c>
+      <c r="B2267" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2267">
+        <v>0</v>
+      </c>
+      <c r="D2267">
+        <v>2145</v>
+      </c>
+      <c r="E2267">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2268" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2268">
+        <v>114</v>
+      </c>
+      <c r="B2268" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2268">
+        <v>0</v>
+      </c>
+      <c r="D2268">
+        <v>3325</v>
+      </c>
+      <c r="E2268">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2269" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2269">
+        <v>114</v>
+      </c>
+      <c r="B2269" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2269">
+        <v>0</v>
+      </c>
+      <c r="D2269">
+        <v>4216</v>
+      </c>
+      <c r="E2269">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2270" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2270">
+        <v>114</v>
+      </c>
+      <c r="B2270" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2270">
+        <v>0</v>
+      </c>
+      <c r="D2270">
+        <v>1609</v>
+      </c>
+      <c r="E2270">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2271" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2271">
+        <v>114</v>
+      </c>
+      <c r="B2271" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2271">
+        <v>0</v>
+      </c>
+      <c r="D2271">
+        <v>2856</v>
+      </c>
+      <c r="E2271">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2272" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2272">
+        <v>114</v>
+      </c>
+      <c r="B2272" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2272">
+        <v>1</v>
+      </c>
+      <c r="D2272">
+        <v>3174</v>
+      </c>
+      <c r="E2272">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2273" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2273">
+        <v>114</v>
+      </c>
+      <c r="B2273" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2273">
+        <v>1</v>
+      </c>
+      <c r="D2273">
+        <v>6979</v>
+      </c>
+      <c r="E2273">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2274" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2274">
+        <v>114</v>
+      </c>
+      <c r="B2274" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2274">
+        <v>1</v>
+      </c>
+      <c r="D2274">
+        <v>7735</v>
+      </c>
+      <c r="E2274">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2275" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2275">
+        <v>114</v>
+      </c>
+      <c r="B2275" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2275">
+        <v>1</v>
+      </c>
+      <c r="D2275">
+        <v>4865</v>
+      </c>
+      <c r="E2275">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2276" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2276">
+        <v>114</v>
+      </c>
+      <c r="B2276" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2276">
+        <v>1</v>
+      </c>
+      <c r="D2276">
+        <v>4056</v>
+      </c>
+      <c r="E2276">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2277" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2277">
+        <v>114</v>
+      </c>
+      <c r="B2277" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2277">
+        <v>1</v>
+      </c>
+      <c r="D2277">
+        <v>5002</v>
+      </c>
+      <c r="E2277">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2278" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2278">
+        <v>114</v>
+      </c>
+      <c r="B2278" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2278">
+        <v>1</v>
+      </c>
+      <c r="D2278">
+        <v>5910</v>
+      </c>
+      <c r="E2278">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2279" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2279">
+        <v>114</v>
+      </c>
+      <c r="B2279" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2279">
+        <v>1</v>
+      </c>
+      <c r="D2279">
+        <v>1668</v>
+      </c>
+      <c r="E2279">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2280" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2280">
+        <v>114</v>
+      </c>
+      <c r="B2280" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2280">
+        <v>1</v>
+      </c>
+      <c r="D2280">
+        <v>2870</v>
+      </c>
+      <c r="E2280">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2281" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2281">
+        <v>114</v>
+      </c>
+      <c r="B2281" s="10">
+        <v>46035</v>
+      </c>
+      <c r="C2281">
+        <v>1</v>
+      </c>
+      <c r="D2281">
+        <v>103</v>
+      </c>
+      <c r="E2281">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
att dia 17 manha
</commit_message>
<xml_diff>
--- a/primeirasemanasetembro.xlsx
+++ b/primeirasemanasetembro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivina\Desktop\jogodobicho\jogodobicho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1ACD559-6130-4A2B-AB80-C065765A727E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{505A374F-8596-4BA7-B272-808215019B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{500AFD6E-13E7-4543-8FDB-D63E104D29D0}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185FBA4-3391-45B3-811A-4861B6CE3709}">
-  <dimension ref="A1:T2321"/>
+  <dimension ref="A1:T2351"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.44140625" customWidth="1"/>
@@ -40798,6 +40798,516 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2322" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2322">
+        <v>117</v>
+      </c>
+      <c r="B2322" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2322">
+        <v>0</v>
+      </c>
+      <c r="D2322">
+        <v>9471</v>
+      </c>
+      <c r="E2322">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2323" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2323">
+        <v>117</v>
+      </c>
+      <c r="B2323" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2323">
+        <v>0</v>
+      </c>
+      <c r="D2323">
+        <v>5902</v>
+      </c>
+      <c r="E2323">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2324" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2324">
+        <v>117</v>
+      </c>
+      <c r="B2324" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2324">
+        <v>0</v>
+      </c>
+      <c r="D2324">
+        <v>5958</v>
+      </c>
+      <c r="E2324">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2325" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2325">
+        <v>117</v>
+      </c>
+      <c r="B2325" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2325">
+        <v>0</v>
+      </c>
+      <c r="D2325">
+        <v>5794</v>
+      </c>
+      <c r="E2325">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2326" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2326">
+        <v>117</v>
+      </c>
+      <c r="B2326" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2326">
+        <v>0</v>
+      </c>
+      <c r="D2326">
+        <v>8434</v>
+      </c>
+      <c r="E2326">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2327" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2327">
+        <v>117</v>
+      </c>
+      <c r="B2327" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2327">
+        <v>0</v>
+      </c>
+      <c r="D2327">
+        <v>9170</v>
+      </c>
+      <c r="E2327">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2328" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2328">
+        <v>117</v>
+      </c>
+      <c r="B2328" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2328">
+        <v>0</v>
+      </c>
+      <c r="D2328">
+        <v>8408</v>
+      </c>
+      <c r="E2328">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2329" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2329">
+        <v>117</v>
+      </c>
+      <c r="B2329" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2329">
+        <v>0</v>
+      </c>
+      <c r="D2329">
+        <v>2593</v>
+      </c>
+      <c r="E2329">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2330" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2330">
+        <v>117</v>
+      </c>
+      <c r="B2330" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2330">
+        <v>0</v>
+      </c>
+      <c r="D2330">
+        <v>3100</v>
+      </c>
+      <c r="E2330">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2331" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2331">
+        <v>117</v>
+      </c>
+      <c r="B2331" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2331">
+        <v>0</v>
+      </c>
+      <c r="D2331">
+        <v>5856</v>
+      </c>
+      <c r="E2331">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2332" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2332">
+        <v>117</v>
+      </c>
+      <c r="B2332" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2332">
+        <v>1</v>
+      </c>
+      <c r="D2332">
+        <v>2371</v>
+      </c>
+      <c r="E2332">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2333" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2333">
+        <v>117</v>
+      </c>
+      <c r="B2333" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2333">
+        <v>1</v>
+      </c>
+      <c r="D2333">
+        <v>4266</v>
+      </c>
+      <c r="E2333">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2334" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2334">
+        <v>117</v>
+      </c>
+      <c r="B2334" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2334">
+        <v>1</v>
+      </c>
+      <c r="D2334">
+        <v>9275</v>
+      </c>
+      <c r="E2334">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2335" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2335">
+        <v>117</v>
+      </c>
+      <c r="B2335" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2335">
+        <v>1</v>
+      </c>
+      <c r="D2335">
+        <v>6352</v>
+      </c>
+      <c r="E2335">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2336" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2336">
+        <v>117</v>
+      </c>
+      <c r="B2336" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2336">
+        <v>1</v>
+      </c>
+      <c r="D2336">
+        <v>4087</v>
+      </c>
+      <c r="E2336">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2337" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2337">
+        <v>117</v>
+      </c>
+      <c r="B2337" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2337">
+        <v>1</v>
+      </c>
+      <c r="D2337">
+        <v>6793</v>
+      </c>
+      <c r="E2337">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2338" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2338">
+        <v>117</v>
+      </c>
+      <c r="B2338" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2338">
+        <v>1</v>
+      </c>
+      <c r="D2338">
+        <v>8109</v>
+      </c>
+      <c r="E2338">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2339" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2339">
+        <v>117</v>
+      </c>
+      <c r="B2339" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2339">
+        <v>1</v>
+      </c>
+      <c r="D2339">
+        <v>101</v>
+      </c>
+      <c r="E2339">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2340" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2340">
+        <v>117</v>
+      </c>
+      <c r="B2340" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2340">
+        <v>1</v>
+      </c>
+      <c r="D2340">
+        <v>6727</v>
+      </c>
+      <c r="E2340">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2341" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2341">
+        <v>117</v>
+      </c>
+      <c r="B2341" s="10">
+        <v>46038</v>
+      </c>
+      <c r="C2341">
+        <v>1</v>
+      </c>
+      <c r="D2341">
+        <v>9688</v>
+      </c>
+      <c r="E2341">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2342" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2342">
+        <v>118</v>
+      </c>
+      <c r="B2342" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2342">
+        <v>0</v>
+      </c>
+      <c r="D2342">
+        <v>4855</v>
+      </c>
+      <c r="E2342">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2343" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2343">
+        <v>118</v>
+      </c>
+      <c r="B2343" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2343">
+        <v>0</v>
+      </c>
+      <c r="D2343">
+        <v>7141</v>
+      </c>
+      <c r="E2343">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2344" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2344">
+        <v>118</v>
+      </c>
+      <c r="B2344" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2344">
+        <v>0</v>
+      </c>
+      <c r="D2344">
+        <v>4432</v>
+      </c>
+      <c r="E2344">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2345" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2345">
+        <v>118</v>
+      </c>
+      <c r="B2345" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2345">
+        <v>0</v>
+      </c>
+      <c r="D2345">
+        <v>2831</v>
+      </c>
+      <c r="E2345">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2346" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2346">
+        <v>118</v>
+      </c>
+      <c r="B2346" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2346">
+        <v>0</v>
+      </c>
+      <c r="D2346">
+        <v>1011</v>
+      </c>
+      <c r="E2346">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2347" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2347">
+        <v>118</v>
+      </c>
+      <c r="B2347" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2347">
+        <v>0</v>
+      </c>
+      <c r="D2347">
+        <v>4041</v>
+      </c>
+      <c r="E2347">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2348" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2348">
+        <v>118</v>
+      </c>
+      <c r="B2348" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2348">
+        <v>0</v>
+      </c>
+      <c r="D2348">
+        <v>6708</v>
+      </c>
+      <c r="E2348">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2349" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2349">
+        <v>118</v>
+      </c>
+      <c r="B2349" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2349">
+        <v>0</v>
+      </c>
+      <c r="D2349">
+        <v>8768</v>
+      </c>
+      <c r="E2349">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2350" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2350">
+        <v>118</v>
+      </c>
+      <c r="B2350" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2350">
+        <v>0</v>
+      </c>
+      <c r="D2350">
+        <v>336</v>
+      </c>
+      <c r="E2350">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2351" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2351">
+        <v>118</v>
+      </c>
+      <c r="B2351" s="10">
+        <v>46039</v>
+      </c>
+      <c r="C2351">
+        <v>0</v>
+      </c>
+      <c r="D2351">
+        <v>2819</v>
+      </c>
+      <c r="E2351">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
att dia 20 manhã
</commit_message>
<xml_diff>
--- a/primeirasemanasetembro.xlsx
+++ b/primeirasemanasetembro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivina\Desktop\jogodobicho\jogodobicho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4B4994-EA3E-4884-AB37-C858A8903C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26941D7-804D-4888-998E-13FCF16E70CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{500AFD6E-13E7-4543-8FDB-D63E104D29D0}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185FBA4-3391-45B3-811A-4861B6CE3709}">
-  <dimension ref="A1:T2361"/>
+  <dimension ref="A1:T2381"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.44140625" customWidth="1"/>
@@ -41478,6 +41478,346 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2362" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2362">
+        <v>119</v>
+      </c>
+      <c r="B2362" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2362">
+        <v>0</v>
+      </c>
+      <c r="D2362">
+        <v>6418</v>
+      </c>
+      <c r="E2362">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2363" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2363">
+        <v>119</v>
+      </c>
+      <c r="B2363" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2363">
+        <v>0</v>
+      </c>
+      <c r="D2363">
+        <v>4211</v>
+      </c>
+      <c r="E2363">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2364" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2364">
+        <v>119</v>
+      </c>
+      <c r="B2364" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2364">
+        <v>0</v>
+      </c>
+      <c r="D2364">
+        <v>1811</v>
+      </c>
+      <c r="E2364">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2365" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2365">
+        <v>119</v>
+      </c>
+      <c r="B2365" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2365">
+        <v>0</v>
+      </c>
+      <c r="D2365">
+        <v>5563</v>
+      </c>
+      <c r="E2365">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2366" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2366">
+        <v>119</v>
+      </c>
+      <c r="B2366" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2366">
+        <v>0</v>
+      </c>
+      <c r="D2366">
+        <v>1821</v>
+      </c>
+      <c r="E2366">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2367" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2367">
+        <v>119</v>
+      </c>
+      <c r="B2367" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2367">
+        <v>0</v>
+      </c>
+      <c r="D2367">
+        <v>9057</v>
+      </c>
+      <c r="E2367">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2368" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2368">
+        <v>119</v>
+      </c>
+      <c r="B2368" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2368">
+        <v>0</v>
+      </c>
+      <c r="D2368">
+        <v>8181</v>
+      </c>
+      <c r="E2368">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2369" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2369">
+        <v>119</v>
+      </c>
+      <c r="B2369" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2369">
+        <v>0</v>
+      </c>
+      <c r="D2369">
+        <v>9671</v>
+      </c>
+      <c r="E2369">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2370" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2370">
+        <v>119</v>
+      </c>
+      <c r="B2370" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2370">
+        <v>0</v>
+      </c>
+      <c r="D2370">
+        <v>8850</v>
+      </c>
+      <c r="E2370">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2371" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2371">
+        <v>119</v>
+      </c>
+      <c r="B2371" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2371">
+        <v>0</v>
+      </c>
+      <c r="D2371">
+        <v>4769</v>
+      </c>
+      <c r="E2371">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2372" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2372">
+        <v>119</v>
+      </c>
+      <c r="B2372" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2372">
+        <v>1</v>
+      </c>
+      <c r="D2372">
+        <v>2915</v>
+      </c>
+      <c r="E2372">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2373" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2373">
+        <v>119</v>
+      </c>
+      <c r="B2373" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2373">
+        <v>1</v>
+      </c>
+      <c r="D2373">
+        <v>8569</v>
+      </c>
+      <c r="E2373">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2374" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2374">
+        <v>119</v>
+      </c>
+      <c r="B2374" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2374">
+        <v>1</v>
+      </c>
+      <c r="D2374">
+        <v>2222</v>
+      </c>
+      <c r="E2374">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2375" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2375">
+        <v>119</v>
+      </c>
+      <c r="B2375" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2375">
+        <v>1</v>
+      </c>
+      <c r="D2375">
+        <v>9331</v>
+      </c>
+      <c r="E2375">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2376" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2376">
+        <v>119</v>
+      </c>
+      <c r="B2376" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2376">
+        <v>1</v>
+      </c>
+      <c r="D2376">
+        <v>5980</v>
+      </c>
+      <c r="E2376">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2377" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2377">
+        <v>119</v>
+      </c>
+      <c r="B2377" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2377">
+        <v>1</v>
+      </c>
+      <c r="D2377">
+        <v>5306</v>
+      </c>
+      <c r="E2377">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2378" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2378">
+        <v>119</v>
+      </c>
+      <c r="B2378" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2378">
+        <v>1</v>
+      </c>
+      <c r="D2378">
+        <v>197</v>
+      </c>
+      <c r="E2378">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2379" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2379">
+        <v>119</v>
+      </c>
+      <c r="B2379" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2379">
+        <v>1</v>
+      </c>
+      <c r="D2379">
+        <v>1371</v>
+      </c>
+      <c r="E2379">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2380" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2380">
+        <v>119</v>
+      </c>
+      <c r="B2380" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2380">
+        <v>1</v>
+      </c>
+      <c r="D2380">
+        <v>358</v>
+      </c>
+      <c r="E2380">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2381" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2381">
+        <v>119</v>
+      </c>
+      <c r="B2381" s="10">
+        <v>46041</v>
+      </c>
+      <c r="C2381">
+        <v>1</v>
+      </c>
+      <c r="D2381">
+        <v>3760</v>
+      </c>
+      <c r="E2381">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
att mes de jan 2026
</commit_message>
<xml_diff>
--- a/primeirasemanasetembro.xlsx
+++ b/primeirasemanasetembro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivina\Desktop\jogodobicho\jogodobicho\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814795FD-2584-4AFD-B0B9-F875308494D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{114750DE-4962-48ED-BE14-8164FC175CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{500AFD6E-13E7-4543-8FDB-D63E104D29D0}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6185FBA4-3391-45B3-811A-4861B6CE3709}">
-  <dimension ref="A1:T2520"/>
+  <dimension ref="A1:T2600"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.44140625" customWidth="1"/>
@@ -44181,6 +44181,1366 @@
         <v>16</v>
       </c>
     </row>
+    <row r="2521" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2521">
+        <v>127</v>
+      </c>
+      <c r="B2521" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2521">
+        <v>0</v>
+      </c>
+      <c r="D2521">
+        <v>7384</v>
+      </c>
+      <c r="E2521">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2522" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2522">
+        <v>127</v>
+      </c>
+      <c r="B2522" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2522">
+        <v>0</v>
+      </c>
+      <c r="D2522">
+        <v>1595</v>
+      </c>
+      <c r="E2522">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2523" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2523">
+        <v>127</v>
+      </c>
+      <c r="B2523" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2523">
+        <v>0</v>
+      </c>
+      <c r="D2523">
+        <v>1221</v>
+      </c>
+      <c r="E2523">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2524" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2524">
+        <v>127</v>
+      </c>
+      <c r="B2524" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2524">
+        <v>0</v>
+      </c>
+      <c r="D2524">
+        <v>9896</v>
+      </c>
+      <c r="E2524">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2525" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2525">
+        <v>127</v>
+      </c>
+      <c r="B2525" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2525">
+        <v>0</v>
+      </c>
+      <c r="D2525">
+        <v>2902</v>
+      </c>
+      <c r="E2525">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2526" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2526">
+        <v>127</v>
+      </c>
+      <c r="B2526" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2526">
+        <v>0</v>
+      </c>
+      <c r="D2526">
+        <v>1602</v>
+      </c>
+      <c r="E2526">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2527" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2527">
+        <v>127</v>
+      </c>
+      <c r="B2527" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2527">
+        <v>0</v>
+      </c>
+      <c r="D2527">
+        <v>4286</v>
+      </c>
+      <c r="E2527">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2528" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2528">
+        <v>127</v>
+      </c>
+      <c r="B2528" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2528">
+        <v>0</v>
+      </c>
+      <c r="D2528">
+        <v>6772</v>
+      </c>
+      <c r="E2528">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2529" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2529">
+        <v>127</v>
+      </c>
+      <c r="B2529" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2529">
+        <v>0</v>
+      </c>
+      <c r="D2529">
+        <v>6380</v>
+      </c>
+      <c r="E2529">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2530" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2530">
+        <v>127</v>
+      </c>
+      <c r="B2530" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2530">
+        <v>0</v>
+      </c>
+      <c r="D2530">
+        <v>9380</v>
+      </c>
+      <c r="E2530">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2531" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2531">
+        <v>127</v>
+      </c>
+      <c r="B2531" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2531">
+        <v>1</v>
+      </c>
+      <c r="D2531">
+        <v>9043</v>
+      </c>
+      <c r="E2531">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2532" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2532">
+        <v>127</v>
+      </c>
+      <c r="B2532" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2532">
+        <v>1</v>
+      </c>
+      <c r="D2532">
+        <v>4709</v>
+      </c>
+      <c r="E2532">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2533" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2533">
+        <v>127</v>
+      </c>
+      <c r="B2533" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2533">
+        <v>1</v>
+      </c>
+      <c r="D2533">
+        <v>9631</v>
+      </c>
+      <c r="E2533">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2534" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2534">
+        <v>127</v>
+      </c>
+      <c r="B2534" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2534">
+        <v>1</v>
+      </c>
+      <c r="D2534">
+        <v>1758</v>
+      </c>
+      <c r="E2534">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2535" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2535">
+        <v>127</v>
+      </c>
+      <c r="B2535" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2535">
+        <v>1</v>
+      </c>
+      <c r="D2535">
+        <v>7218</v>
+      </c>
+      <c r="E2535">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2536" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2536">
+        <v>127</v>
+      </c>
+      <c r="B2536" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2536">
+        <v>1</v>
+      </c>
+      <c r="D2536">
+        <v>2620</v>
+      </c>
+      <c r="E2536">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2537" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2537">
+        <v>127</v>
+      </c>
+      <c r="B2537" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2537">
+        <v>1</v>
+      </c>
+      <c r="D2537">
+        <v>2966</v>
+      </c>
+      <c r="E2537">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2538" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2538">
+        <v>127</v>
+      </c>
+      <c r="B2538" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2538">
+        <v>1</v>
+      </c>
+      <c r="D2538">
+        <v>2611</v>
+      </c>
+      <c r="E2538">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2539" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2539">
+        <v>127</v>
+      </c>
+      <c r="B2539" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2539">
+        <v>1</v>
+      </c>
+      <c r="D2539">
+        <v>5596</v>
+      </c>
+      <c r="E2539">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2540" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2540">
+        <v>127</v>
+      </c>
+      <c r="B2540" s="10">
+        <v>46050</v>
+      </c>
+      <c r="C2540">
+        <v>1</v>
+      </c>
+      <c r="D2540">
+        <v>3092</v>
+      </c>
+      <c r="E2540">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2541" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2541">
+        <v>128</v>
+      </c>
+      <c r="B2541" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2541">
+        <v>0</v>
+      </c>
+      <c r="D2541">
+        <v>6346</v>
+      </c>
+      <c r="E2541">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2542" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2542">
+        <v>128</v>
+      </c>
+      <c r="B2542" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2542">
+        <v>0</v>
+      </c>
+      <c r="D2542">
+        <v>9722</v>
+      </c>
+      <c r="E2542">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2543" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2543">
+        <v>128</v>
+      </c>
+      <c r="B2543" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2543">
+        <v>0</v>
+      </c>
+      <c r="D2543">
+        <v>6666</v>
+      </c>
+      <c r="E2543">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2544" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2544">
+        <v>128</v>
+      </c>
+      <c r="B2544" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2544">
+        <v>0</v>
+      </c>
+      <c r="D2544">
+        <v>8204</v>
+      </c>
+      <c r="E2544">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2545" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2545">
+        <v>128</v>
+      </c>
+      <c r="B2545" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2545">
+        <v>0</v>
+      </c>
+      <c r="D2545">
+        <v>9273</v>
+      </c>
+      <c r="E2545">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2546" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2546">
+        <v>128</v>
+      </c>
+      <c r="B2546" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2546">
+        <v>0</v>
+      </c>
+      <c r="D2546">
+        <v>65</v>
+      </c>
+      <c r="E2546">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2547" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2547">
+        <v>128</v>
+      </c>
+      <c r="B2547" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2547">
+        <v>0</v>
+      </c>
+      <c r="D2547">
+        <v>6085</v>
+      </c>
+      <c r="E2547">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2548" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2548">
+        <v>128</v>
+      </c>
+      <c r="B2548" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2548">
+        <v>0</v>
+      </c>
+      <c r="D2548">
+        <v>8956</v>
+      </c>
+      <c r="E2548">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2549" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2549">
+        <v>128</v>
+      </c>
+      <c r="B2549" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2549">
+        <v>0</v>
+      </c>
+      <c r="D2549">
+        <v>6712</v>
+      </c>
+      <c r="E2549">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2550" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2550">
+        <v>128</v>
+      </c>
+      <c r="B2550" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2550">
+        <v>0</v>
+      </c>
+      <c r="D2550">
+        <v>2478</v>
+      </c>
+      <c r="E2550">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2551" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2551">
+        <v>128</v>
+      </c>
+      <c r="B2551" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2551">
+        <v>1</v>
+      </c>
+      <c r="D2551">
+        <v>9753</v>
+      </c>
+      <c r="E2551">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2552" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2552">
+        <v>128</v>
+      </c>
+      <c r="B2552" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2552">
+        <v>1</v>
+      </c>
+      <c r="D2552">
+        <v>4687</v>
+      </c>
+      <c r="E2552">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2553" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2553">
+        <v>128</v>
+      </c>
+      <c r="B2553" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2553">
+        <v>1</v>
+      </c>
+      <c r="D2553">
+        <v>9515</v>
+      </c>
+      <c r="E2553">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2554" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2554">
+        <v>128</v>
+      </c>
+      <c r="B2554" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2554">
+        <v>1</v>
+      </c>
+      <c r="D2554">
+        <v>5996</v>
+      </c>
+      <c r="E2554">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2555" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2555">
+        <v>128</v>
+      </c>
+      <c r="B2555" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2555">
+        <v>1</v>
+      </c>
+      <c r="D2555">
+        <v>6303</v>
+      </c>
+      <c r="E2555">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2556" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2556">
+        <v>128</v>
+      </c>
+      <c r="B2556" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2556">
+        <v>1</v>
+      </c>
+      <c r="D2556">
+        <v>9258</v>
+      </c>
+      <c r="E2556">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2557" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2557">
+        <v>128</v>
+      </c>
+      <c r="B2557" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2557">
+        <v>1</v>
+      </c>
+      <c r="D2557">
+        <v>436</v>
+      </c>
+      <c r="E2557">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2558" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2558">
+        <v>128</v>
+      </c>
+      <c r="B2558" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2558">
+        <v>1</v>
+      </c>
+      <c r="D2558">
+        <v>620</v>
+      </c>
+      <c r="E2558">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2559" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2559">
+        <v>128</v>
+      </c>
+      <c r="B2559" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2559">
+        <v>1</v>
+      </c>
+      <c r="D2559">
+        <v>9008</v>
+      </c>
+      <c r="E2559">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2560" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2560">
+        <v>128</v>
+      </c>
+      <c r="B2560" s="10">
+        <v>46051</v>
+      </c>
+      <c r="C2560">
+        <v>1</v>
+      </c>
+      <c r="D2560">
+        <v>7080</v>
+      </c>
+      <c r="E2560">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2561" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2561">
+        <v>129</v>
+      </c>
+      <c r="B2561" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2561">
+        <v>0</v>
+      </c>
+      <c r="D2561">
+        <v>9172</v>
+      </c>
+      <c r="E2561">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2562" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2562">
+        <v>129</v>
+      </c>
+      <c r="B2562" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2562">
+        <v>0</v>
+      </c>
+      <c r="D2562">
+        <v>1368</v>
+      </c>
+      <c r="E2562">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2563" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2563">
+        <v>129</v>
+      </c>
+      <c r="B2563" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2563">
+        <v>0</v>
+      </c>
+      <c r="D2563">
+        <v>7720</v>
+      </c>
+      <c r="E2563">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2564" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2564">
+        <v>129</v>
+      </c>
+      <c r="B2564" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2564">
+        <v>0</v>
+      </c>
+      <c r="D2564">
+        <v>1622</v>
+      </c>
+      <c r="E2564">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2565" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2565">
+        <v>129</v>
+      </c>
+      <c r="B2565" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2565">
+        <v>0</v>
+      </c>
+      <c r="D2565">
+        <v>8306</v>
+      </c>
+      <c r="E2565">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2566" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2566">
+        <v>129</v>
+      </c>
+      <c r="B2566" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2566">
+        <v>0</v>
+      </c>
+      <c r="D2566">
+        <v>2227</v>
+      </c>
+      <c r="E2566">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2567" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2567">
+        <v>129</v>
+      </c>
+      <c r="B2567" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2567">
+        <v>0</v>
+      </c>
+      <c r="D2567">
+        <v>9527</v>
+      </c>
+      <c r="E2567">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2568" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2568">
+        <v>129</v>
+      </c>
+      <c r="B2568" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2568">
+        <v>0</v>
+      </c>
+      <c r="D2568">
+        <v>6534</v>
+      </c>
+      <c r="E2568">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2569" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2569">
+        <v>129</v>
+      </c>
+      <c r="B2569" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2569">
+        <v>0</v>
+      </c>
+      <c r="D2569">
+        <v>7564</v>
+      </c>
+      <c r="E2569">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2570" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2570">
+        <v>129</v>
+      </c>
+      <c r="B2570" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2570">
+        <v>0</v>
+      </c>
+      <c r="D2570">
+        <v>4182</v>
+      </c>
+      <c r="E2570">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2571" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2571">
+        <v>129</v>
+      </c>
+      <c r="B2571" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2571">
+        <v>1</v>
+      </c>
+      <c r="D2571">
+        <v>3248</v>
+      </c>
+      <c r="E2571">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2572" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2572">
+        <v>129</v>
+      </c>
+      <c r="B2572" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2572">
+        <v>1</v>
+      </c>
+      <c r="D2572">
+        <v>211</v>
+      </c>
+      <c r="E2572">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2573" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2573">
+        <v>129</v>
+      </c>
+      <c r="B2573" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2573">
+        <v>1</v>
+      </c>
+      <c r="D2573">
+        <v>1817</v>
+      </c>
+      <c r="E2573">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2574" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2574">
+        <v>129</v>
+      </c>
+      <c r="B2574" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2574">
+        <v>1</v>
+      </c>
+      <c r="D2574">
+        <v>244</v>
+      </c>
+      <c r="E2574">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2575" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2575">
+        <v>129</v>
+      </c>
+      <c r="B2575" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2575">
+        <v>1</v>
+      </c>
+      <c r="D2575">
+        <v>8190</v>
+      </c>
+      <c r="E2575">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2576" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2576">
+        <v>129</v>
+      </c>
+      <c r="B2576" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2576">
+        <v>1</v>
+      </c>
+      <c r="D2576">
+        <v>1360</v>
+      </c>
+      <c r="E2576">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2577" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2577">
+        <v>129</v>
+      </c>
+      <c r="B2577" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2577">
+        <v>1</v>
+      </c>
+      <c r="D2577">
+        <v>4335</v>
+      </c>
+      <c r="E2577">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2578" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2578">
+        <v>129</v>
+      </c>
+      <c r="B2578" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2578">
+        <v>1</v>
+      </c>
+      <c r="D2578">
+        <v>7017</v>
+      </c>
+      <c r="E2578">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2579" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2579">
+        <v>129</v>
+      </c>
+      <c r="B2579" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2579">
+        <v>1</v>
+      </c>
+      <c r="D2579">
+        <v>1445</v>
+      </c>
+      <c r="E2579">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2580" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2580">
+        <v>129</v>
+      </c>
+      <c r="B2580" s="10">
+        <v>46052</v>
+      </c>
+      <c r="C2580">
+        <v>1</v>
+      </c>
+      <c r="D2580">
+        <v>1476</v>
+      </c>
+      <c r="E2580">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2581" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2581">
+        <v>130</v>
+      </c>
+      <c r="B2581" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2581">
+        <v>0</v>
+      </c>
+      <c r="D2581">
+        <v>2457</v>
+      </c>
+      <c r="E2581">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2582" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2582">
+        <v>130</v>
+      </c>
+      <c r="B2582" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2582">
+        <v>0</v>
+      </c>
+      <c r="D2582">
+        <v>6296</v>
+      </c>
+      <c r="E2582">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2583" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2583">
+        <v>130</v>
+      </c>
+      <c r="B2583" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2583">
+        <v>0</v>
+      </c>
+      <c r="D2583">
+        <v>7873</v>
+      </c>
+      <c r="E2583">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2584" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2584">
+        <v>130</v>
+      </c>
+      <c r="B2584" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2584">
+        <v>0</v>
+      </c>
+      <c r="D2584">
+        <v>4926</v>
+      </c>
+      <c r="E2584">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2585" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2585">
+        <v>130</v>
+      </c>
+      <c r="B2585" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2585">
+        <v>0</v>
+      </c>
+      <c r="D2585">
+        <v>3125</v>
+      </c>
+      <c r="E2585">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2586" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2586">
+        <v>130</v>
+      </c>
+      <c r="B2586" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2586">
+        <v>0</v>
+      </c>
+      <c r="D2586">
+        <v>9687</v>
+      </c>
+      <c r="E2586">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2587" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2587">
+        <v>130</v>
+      </c>
+      <c r="B2587" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2587">
+        <v>0</v>
+      </c>
+      <c r="D2587">
+        <v>2379</v>
+      </c>
+      <c r="E2587">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2588" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2588">
+        <v>130</v>
+      </c>
+      <c r="B2588" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2588">
+        <v>0</v>
+      </c>
+      <c r="D2588">
+        <v>8508</v>
+      </c>
+      <c r="E2588">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2589" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2589">
+        <v>130</v>
+      </c>
+      <c r="B2589" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2589">
+        <v>0</v>
+      </c>
+      <c r="D2589">
+        <v>6188</v>
+      </c>
+      <c r="E2589">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2590" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2590">
+        <v>130</v>
+      </c>
+      <c r="B2590" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2590">
+        <v>0</v>
+      </c>
+      <c r="D2590">
+        <v>1888</v>
+      </c>
+      <c r="E2590">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2591" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2591">
+        <v>130</v>
+      </c>
+      <c r="B2591" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2591">
+        <v>1</v>
+      </c>
+      <c r="D2591">
+        <v>295</v>
+      </c>
+      <c r="E2591">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2592" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2592">
+        <v>130</v>
+      </c>
+      <c r="B2592" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2592">
+        <v>1</v>
+      </c>
+      <c r="D2592">
+        <v>6984</v>
+      </c>
+      <c r="E2592">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2593" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2593">
+        <v>130</v>
+      </c>
+      <c r="B2593" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2593">
+        <v>1</v>
+      </c>
+      <c r="D2593">
+        <v>8710</v>
+      </c>
+      <c r="E2593">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2594" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2594">
+        <v>130</v>
+      </c>
+      <c r="B2594" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2594">
+        <v>1</v>
+      </c>
+      <c r="D2594">
+        <v>870</v>
+      </c>
+      <c r="E2594">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2595" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2595">
+        <v>130</v>
+      </c>
+      <c r="B2595" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2595">
+        <v>1</v>
+      </c>
+      <c r="D2595">
+        <v>8206</v>
+      </c>
+      <c r="E2595">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2596" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2596">
+        <v>130</v>
+      </c>
+      <c r="B2596" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2596">
+        <v>1</v>
+      </c>
+      <c r="D2596">
+        <v>1928</v>
+      </c>
+      <c r="E2596">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2597" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2597">
+        <v>130</v>
+      </c>
+      <c r="B2597" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2597">
+        <v>1</v>
+      </c>
+      <c r="D2597">
+        <v>8451</v>
+      </c>
+      <c r="E2597">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2598" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2598">
+        <v>130</v>
+      </c>
+      <c r="B2598" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2598">
+        <v>1</v>
+      </c>
+      <c r="D2598">
+        <v>6326</v>
+      </c>
+      <c r="E2598">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2599" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2599">
+        <v>130</v>
+      </c>
+      <c r="B2599" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2599">
+        <v>1</v>
+      </c>
+      <c r="D2599">
+        <v>4344</v>
+      </c>
+      <c r="E2599">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2600" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2600">
+        <v>130</v>
+      </c>
+      <c r="B2600" s="10">
+        <v>46053</v>
+      </c>
+      <c r="C2600">
+        <v>1</v>
+      </c>
+      <c r="D2600">
+        <v>3515</v>
+      </c>
+      <c r="E2600">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>